<commit_message>
Fix tracker footnote dropped during recalculation, clean remaining dashes
- Restore row 13's "how to add a new activity" footnote and its merge,
  lost when the LibreOffice recalculation attempt touched the file
- Drop stray column-width metadata left over from the old F-J columns
- Replace remaining em/en dashes in the tracker and app/index.html footer
</commit_message>
<xml_diff>
--- a/Performance_Tracker.xlsx
+++ b/Performance_Tracker.xlsx
@@ -112,15 +112,6 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -137,6 +128,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -409,190 +407,189 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="9"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="9" min="1" max="1"/>
+    <col width="22" customWidth="1" style="9" min="2" max="2"/>
+    <col width="24" customWidth="1" style="9" min="3" max="3"/>
+    <col width="26" customWidth="1" style="9" min="4" max="4"/>
+    <col width="12" customWidth="1" style="9" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>TPS_3371_TEAM_20 — Team Contribution &amp; Performance Tracker</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="27.75" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Team Lead: Peter  |  Score = 0–100 per activity, based on actual participation/contribution  |  Yellow cells = enter scores  |  Column header = Date – Activity Type: Brief description  |  Not an official course grade  |  Keep accurate — instructor reviews repo activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="1" ht="25.5" customHeight="1" s="9">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>TPS_3371_TEAM_20 - Team Contribution &amp; Performance Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.75" customHeight="1" s="9">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Team Lead: Peter  |  Score = 0-100 per activity, based on actual participation/contribution  |  Yellow cells = enter scores  |  Column header = Date - Activity Type: Brief description  |  Not an official course grade  |  Keep accurate - instructor reviews repo activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" s="9">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Team Member</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Milestone 1 (Week 3): Project Proposal</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Week 6 Group Exercise Pack: Team Activity</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Week 6 Group Exercise Pack: Individual Assignment</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Peter</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E5" s="8">
+      <c r="B5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" s="5">
         <f>IFERROR(AVERAGE(B5:D5),"")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Daja</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E6" s="8">
+      <c r="B6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="5">
         <f>IFERROR(AVERAGE(B6:D6),"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sophia</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E7" s="8">
+      <c r="B7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="5">
         <f>IFERROR(AVERAGE(B7:D7),"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Elizabeth</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E8" s="8">
+      <c r="B8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" s="5">
         <f>IFERROR(AVERAGE(B8:D8),"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Yoki</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E9" s="8">
+      <c r="B9" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="5">
         <f>IFERROR(AVERAGE(B9:D9),"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Team Average</t>
         </is>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="7">
         <f>IFERROR(AVERAGE(B5:B9),"")</f>
         <v/>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="7">
         <f>IFERROR(AVERAGE(C5:C9),"")</f>
         <v/>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="7">
         <f>IFERROR(AVERAGE(D5:D9),"")</f>
         <v/>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="7">
         <f>IFERROR(AVERAGE(E5:E9),"")</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>To add a new activity: insert a column before "Average", title it "[Date] – [Type]: [Brief description]" (e.g., "Sep 22 – Out-of-Class: Data Dictionary Draft"), then enter each member's score 0–100.</t>
+    <row r="13" ht="15" customHeight="1" s="9">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>To add a new activity: insert a column before "Average", title it "[Date] - [Type]: [Brief description]" (e.g., "Sep 22 - Out-of-Class: Data Dictionary Draft"), then enter each member's score 0-100.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:I9">
     <cfRule type="expression" priority="2" dxfId="0">

</xml_diff>

<commit_message>
Add Milestone 2 and Week 8 columns to the performance tracker
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Performance_Tracker.xlsx
+++ b/Performance_Tracker.xlsx
@@ -404,14 +404,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="9" min="1" max="1"/>
     <col width="22" customWidth="1" style="9" min="2" max="2"/>
     <col width="24" customWidth="1" style="9" min="3" max="3"/>
     <col width="26" customWidth="1" style="9" min="4" max="4"/>
-    <col width="12" customWidth="1" style="9" min="5" max="5"/>
+    <col width="26" customWidth="1" style="9" min="5" max="5"/>
+    <col width="24" customWidth="1" style="9" min="6" max="6"/>
+    <col width="12" customWidth="1" style="9" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="9">
@@ -420,6 +422,12 @@
           <t>TPS_3371_TEAM_20 - Team Contribution &amp; Performance Tracker</t>
         </is>
       </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2" ht="27.75" customHeight="1" s="9">
       <c r="A2" s="10" t="inlineStr">
@@ -427,7 +435,14 @@
           <t>Team Lead: Peter  |  Score = 0-100 per activity, based on actual participation/contribution  |  Yellow cells = enter scores  |  Column header = Date - Activity Type: Brief description  |  Not an official course grade  |  Keep accurate - instructor reviews repo activity</t>
         </is>
       </c>
-    </row>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+    </row>
+    <row r="3"/>
     <row r="4" ht="60" customHeight="1" s="9">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -451,6 +466,16 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Milestone 2 (Weeks 4-7): Client-Side System</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Week 8 Team Activity: Local Backend</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Average</t>
         </is>
       </c>
@@ -470,8 +495,14 @@
       <c r="D5" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E5" s="5">
-        <f>IFERROR(AVERAGE(B5:D5),"")</f>
+      <c r="E5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="5">
+        <f>IFERROR(AVERAGE(B5:F5),"")</f>
         <v/>
       </c>
     </row>
@@ -490,8 +521,14 @@
       <c r="D6" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E6" s="5">
-        <f>IFERROR(AVERAGE(B6:D6),"")</f>
+      <c r="E6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="5">
+        <f>IFERROR(AVERAGE(B6:F6),"")</f>
         <v/>
       </c>
     </row>
@@ -510,8 +547,14 @@
       <c r="D7" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E7" s="5">
-        <f>IFERROR(AVERAGE(B7:D7),"")</f>
+      <c r="E7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="5">
+        <f>IFERROR(AVERAGE(B7:F7),"")</f>
         <v/>
       </c>
     </row>
@@ -530,8 +573,14 @@
       <c r="D8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E8" s="5">
-        <f>IFERROR(AVERAGE(B8:D8),"")</f>
+      <c r="E8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="5">
+        <f>IFERROR(AVERAGE(B8:F8),"")</f>
         <v/>
       </c>
     </row>
@@ -550,11 +599,18 @@
       <c r="D9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E9" s="5">
-        <f>IFERROR(AVERAGE(B9:D9),"")</f>
-        <v/>
-      </c>
-    </row>
+      <c r="E9" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="5">
+        <f>IFERROR(AVERAGE(B9:F9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -577,19 +633,34 @@
         <f>IFERROR(AVERAGE(E5:E9),"")</f>
         <v/>
       </c>
-    </row>
+      <c r="F11" s="7">
+        <f>IFERROR(AVERAGE(F5:F9),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="7">
+        <f>IFERROR(AVERAGE(G5:G9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="9">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>To add a new activity: insert a column before "Average", title it "[Date] - [Type]: [Brief description]" (e.g., "Sep 22 - Out-of-Class: Data Dictionary Draft"), then enter each member's score 0-100.</t>
         </is>
       </c>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:I9">
     <cfRule type="expression" priority="2" dxfId="0">

</xml_diff>